<commit_message>
Fix the three unit tests Person feed 1 broke (platform validation 5)
- resolve_feed: when a provider name matches several Rules documents (SEC
  submissions feed Company and Person), the one that acquires the feed
  answers; a clear error when none or several do.
- Mapping Document words: token_match@1 and name_shape@1 in plain words; a
  negated condition shows as NOT (...); excluded words are named; a ceiling
  of 1 or more is shown. Company's workbooks are unchanged; Person's were
  regenerated with rules mapdoc write.
- The pinned Mapping Document set includes Person's two.

Operator: "yes" to these code fixes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UBWe8qUSEPzmhbtUpEQ7d5
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/person.xlsx
+++ b/rules/merge/kinds/person.xlsx
@@ -759,7 +759,7 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>token_match@1 field: name; normalizer: conformed; token_list: entity_legal_form; min_count: 1; max_count: 1; and name_shape@1 field: name; normalizer: conformed; min_tokens: 2; max_tokens: 5; suffix_list: person_suffix; forbid_digits: value: True; applies_to: raw; forbid_characters: value: &amp;; applies_to: raw; and structural_fields is empty</t>
+          <t>name holds at least 1 and at most 1 word(s) of the list entity_legal_form; and name is shaped like a person's name: 2 to 5 words, no digits or forbidden characters (suffixes from person_suffix allowed); and structural_fields is empty</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -797,7 +797,7 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>token_match@1 field: name; normalizer: conformed; token_list: entity_legal_form; exclude_list: ambiguous; min_count: 1</t>
+          <t>name holds at least 1 word(s) of the list entity_legal_form (not counting ambiguous)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -835,7 +835,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>token_match@1 field: name; normalizer: conformed; token_list: entity_legal_form; min_count: 1; and structural_fields is empty; and name_shape@1 field: name; normalizer: conformed; min_tokens: 2; max_tokens: 5; suffix_list: person_suffix; forbid_digits: value: True; applies_to: raw; forbid_characters: value: &amp;; applies_to: raw</t>
+          <t>NOT (name holds at least 1 word(s) of the list entity_legal_form); and structural_fields is empty; and name is shaped like a person's name: 2 to 5 words, no digits or forbidden characters (suffixes from person_suffix allowed)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
SEC ownership: the reporting owner's Dataset Contract (draft, not switched on)
- The owner table carries the filing's issuer CIK and period of report, so
  the owner's link to the issuer is dated by the filing.
- sec.ownership.reporting_owner.v1: one owner on one filing, a Person when
  the name is person-shaped and the filing names it a director or officer;
  EMPLOYED_BY (director, officer) and BENEFICIAL_OWNER_OF (ten-percent owner)
  as dated sightings to the issuer's Company.
- Person rules: sec-ownership-person and sec-ownership-person-cik, declared,
  not switched on. Measured: 4,622 of 4,622 labelled people, 0 of 363
  entities called a person.
- The Proving Run stops on the Merge Stage's closure limit; a separate fix.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoWChUCsVyST73AjRcdH6D
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/person.xlsx
+++ b/rules/merge/kinds/person.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>person-2026-09-30.1</t>
+          <t>person-2026-10-13.1</t>
         </is>
       </c>
     </row>
@@ -505,11 +505,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -544,6 +544,23 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/person.yaml defaults.sources[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml defaults.sources[1]</t>
         </is>
       </c>
     </row>
@@ -562,7 +579,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="61" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
@@ -603,7 +620,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.person.v1</t>
+          <t>sec.submissions.person.v1, sec.ownership.reporting_owner.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -633,12 +650,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -879,6 +896,196 @@
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/person.yaml rules[0].steps[4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2-guard</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>rpt_owner_name holds at least 1 and at most 1 word(s) of the list entity_legal_form; and rpt_owner_name is shaped like a person's name: 2 to 5 words, no digits or forbidden characters (suffixes from person_suffix allowed)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[2].steps[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>entity_undetermined</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>rpt_owner_name holds at least 1 word(s) of the list entity_legal_form (not counting ambiguous)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[2].steps[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>3-director</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>NOT (rpt_owner_name holds at least 1 word(s) of the list entity_legal_form); and rpt_owner_name is shaped like a person's name: 2 to 5 words, no digits or forbidden characters (suffixes from person_suffix allowed); and is_director is one of: True</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[2].steps[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>3-officer</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>NOT (rpt_owner_name holds at least 1 word(s) of the list entity_legal_form); and rpt_owner_name is shaped like a person's name: 2 to 5 words, no digits or forbidden characters (suffixes from person_suffix allowed); and is_officer is one of: True</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[2].steps[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Otherwise</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[2].steps[4]</t>
         </is>
       </c>
     </row>
@@ -893,13 +1100,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="62" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -983,6 +1190,44 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/person.yaml rules[1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>sec-ownership-person-cik</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13.1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>sec.ownership.reporting_owner.v1</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>The record's CIK is the one a Company holds; and Exactly one Company holds that CIK, or none</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/person.yaml rules[3]</t>
         </is>
       </c>
     </row>

</xml_diff>